<commit_message>
fix upload master data
Root cause & fix:

Sebelum	Sesudah
Strategy	upsert dengan onConflict: 'lower(po_number),...'	Insert biasa + dedup check di client
Error	PostgREST reject ekspresi lower() di onConflict	Tidak ada — pakai .in() query + Set key comparison
Duplikat	Bergantung DB constraint expression	Filter di JS: key = po_number|receive_date|material_name|receive_number|batch_size
Batch	Single upsert	Loop 200 baris per batch
</commit_message>
<xml_diff>
--- a/Support Data/ADF_QC_LAB_RAW_MATERIAL_REPORT_RPT_ADF_LAB_RAW_MATERIAL_LAYOUT - 2026-07-16T105438.459.xlsx
+++ b/Support Data/ADF_QC_LAB_RAW_MATERIAL_REPORT_RPT_ADF_LAB_RAW_MATERIAL_LAYOUT - 2026-07-16T105438.459.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
@@ -10,8 +10,8 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="page\x2dtotal">Sheet1!$A$10</definedName>
-    <definedName name="page\x2dtotal\x2dmaster0">Sheet1!$A$10</definedName>
+    <definedName name="page\x2dtotal">Sheet1!$A$9</definedName>
+    <definedName name="page\x2dtotal\x2dmaster0">Sheet1!$A$9</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -964,29 +964,29 @@
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1334,7 +1334,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:R10"/>
+  <dimension ref="A1:R9"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.047619047619" customWidth="1"/>
@@ -1355,420 +1355,409 @@
     <col min="18" max="18" width="20.5714285714286" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
+    <row r="1" ht="15.75" spans="1:18">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="3"/>
+      <c r="J1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="2" ht="15.75" spans="1:18">
-      <c r="A2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I2" s="4"/>
-      <c r="J2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>16</v>
+    <row r="2" ht="33.75" spans="1:18">
+      <c r="A2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="5"/>
+      <c r="F2" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I2" s="7"/>
+      <c r="J2" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>32</v>
       </c>
     </row>
-    <row r="3" ht="33.75" spans="1:18">
-      <c r="A3" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="5" t="s">
+    <row r="3" ht="45" spans="1:18">
+      <c r="A3" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E3" s="6"/>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="I3" s="7"/>
+      <c r="J3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="O3" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q3" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="R3" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" ht="33.75" spans="1:18">
+      <c r="A4" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" s="5"/>
+      <c r="F4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" s="8"/>
-      <c r="J3" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="L3" s="5" t="s">
+      <c r="G4" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="I4" s="7"/>
+      <c r="J4" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="L4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="M3" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="O3" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="P3" s="5" t="s">
+      <c r="M4" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="N4" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="O4" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="P4" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="Q3" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="R3" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" ht="45" spans="1:18">
-      <c r="A4" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="I4" s="8"/>
-      <c r="J4" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="K4" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="L4" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="M4" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="N4" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="O4" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="P4" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q4" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="R4" s="5" t="s">
+      <c r="Q4" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="R4" s="4" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="5" ht="33.75" spans="1:18">
-      <c r="A5" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C5" s="5" t="s">
+      <c r="A5" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="I5" s="7"/>
+      <c r="J5" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="M5" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="P5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q5" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="R5" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" ht="45" spans="1:18">
+      <c r="A6" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="6"/>
-      <c r="F5" s="5" t="s">
+      <c r="E6" s="5"/>
+      <c r="F6" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="G5" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="I5" s="8"/>
-      <c r="J5" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="K5" s="5" t="s">
+      <c r="G6" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="I6" s="7"/>
+      <c r="J6" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K6" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="L5" s="5" t="s">
+      <c r="L6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="M5" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="N5" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="O5" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="P5" s="5" t="s">
+      <c r="M6" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="N6" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="O6" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="P6" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="Q5" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="R5" s="5" t="s">
+      <c r="Q6" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="R6" s="4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="6" ht="33.75" spans="1:18">
-      <c r="A6" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C6" s="5" t="s">
+    <row r="7" ht="56.25" spans="1:18">
+      <c r="A7" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D7" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E7" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F7" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="G6" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="I6" s="8"/>
-      <c r="J6" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="L6" s="5" t="s">
+      <c r="G7" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="I7" s="7"/>
+      <c r="J7" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="L7" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="M6" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="N6" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="O6" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="P6" s="5" t="s">
+      <c r="M7" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="N7" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="O7" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="P7" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="Q6" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="R6" s="5" t="s">
+      <c r="Q7" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="R7" s="4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="7" ht="45" spans="1:18">
-      <c r="A7" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="E7" s="6"/>
-      <c r="F7" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="I7" s="8"/>
-      <c r="J7" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="L7" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="M7" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="N7" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="O7" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="P7" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q7" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="R7" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="8" ht="56.25" spans="1:18">
-      <c r="A8" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="I8" s="8"/>
-      <c r="J8" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="K8" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="L8" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="M8" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="N8" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="O8" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="P8" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q8" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="R8" s="5" t="s">
-        <v>32</v>
-      </c>
+    <row r="8" spans="1:18">
+      <c r="A8" s="8"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
     </row>
     <row r="9" spans="1:18">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-    </row>
-    <row r="10" spans="1:18">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
+      <c r="A9" s="8"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A1:H1"/>
+  <mergeCells count="9">
+    <mergeCell ref="H1:I1"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="H3:I3"/>
     <mergeCell ref="H4:I4"/>
     <mergeCell ref="H5:I5"/>
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="A8:H8"/>
     <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A10:H10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>